<commit_message>
Añadir métricas DataForSEO (autoridad, indexadas, backlinks, spam) y recomendación basada en datos
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WDJpcdhdbSFMwa1eDYh7n7
</commit_message>
<xml_diff>
--- a/Inventario_de_Hosting_Instagram_SEO.xlsx
+++ b/Inventario_de_Hosting_Instagram_SEO.xlsx
@@ -8,6 +8,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="HOSTINGS " sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="INSTAGRAMS " sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="NOTAS MÉTRICAS" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -137,7 +138,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -208,6 +209,21 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -443,9 +459,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Hostings" displayName="Hostings" ref="A2:H71" headerRowCount="1" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
-  <autoFilter ref="A2:H71"/>
-  <tableColumns count="8">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Hostings" displayName="Hostings" ref="A2:M71" headerRowCount="1" totalsRowShown="0" headerRowDxfId="16" dataDxfId="15">
+  <autoFilter ref="A2:M71"/>
+  <tableColumns count="13">
     <tableColumn id="1" name="#" dataDxfId="14">
       <calculatedColumnFormula array="1">ROW()-ROW(Hostings[#Headers])</calculatedColumnFormula>
     </tableColumn>
@@ -458,6 +474,11 @@
     <tableColumn id="6" name="Recomendación SEO"/>
     <tableColumn id="7" name="Motivo"/>
     <tableColumn id="8" name="Datos a verificar"/>
+    <tableColumn id="9" name="Autoridad (0-100)"/>
+    <tableColumn id="10" name="URLs indexadas (Google)"/>
+    <tableColumn id="11" name="Backlinks"/>
+    <tableColumn id="12" name="Dominios de referencia"/>
+    <tableColumn id="13" name="Spam score"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium15" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -798,7 +819,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H78"/>
+  <dimension ref="A1:M78"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
   <cols>
     <col width="5.75" customWidth="1" min="1" max="1"/>
@@ -806,8 +827,13 @@
     <col width="28.25" customWidth="1" min="3" max="3"/>
     <col width="15.75" customWidth="1" min="4" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
-    <col width="70" customWidth="1" min="7" max="7"/>
-    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="80" customWidth="1" min="7" max="7"/>
+    <col width="34" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="14" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="21" customHeight="1">
@@ -858,6 +884,31 @@
           <t>Datos a verificar</t>
         </is>
       </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>Autoridad (0-100)</t>
+        </is>
+      </c>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>URLs indexadas (Google)</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>Backlinks</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Dominios de referencia</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>Spam score</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="19.9" customHeight="1">
       <c r="A3" s="7">
@@ -890,13 +941,28 @@
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>Marca principal, dominio exacto del negocio</t>
+          <t>Marca principal. Autoridad baja y casi sin indexar (1): revisar SEO técnico, pero es la marca</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>spam alto: revisar/desautorizar enlaces</t>
+        </is>
+      </c>
+      <c r="I3" s="25" t="n">
+        <v>21</v>
+      </c>
+      <c r="J3" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="K3" s="25" t="n">
+        <v>2687</v>
+      </c>
+      <c r="L3" s="25" t="n">
+        <v>2526</v>
+      </c>
+      <c r="M3" s="26" t="n">
+        <v>53</v>
       </c>
     </row>
     <row r="4" ht="19.9" customHeight="1">
@@ -930,13 +996,24 @@
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
-          <t>Marca de alto tráfico y búsquedas de marca; sostiene subdominios activos</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Marca de alto tráfico: 705 URLs indexadas, 3.1k dominios ref., sostiene subdominios activos</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr"/>
+      <c r="I4" s="25" t="n">
+        <v>31</v>
+      </c>
+      <c r="J4" s="25" t="n">
+        <v>705</v>
+      </c>
+      <c r="K4" s="25" t="n">
+        <v>3769</v>
+      </c>
+      <c r="L4" s="25" t="n">
+        <v>3087</v>
+      </c>
+      <c r="M4" s="25" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="5" ht="19.9" customHeight="1">
@@ -974,6 +1051,11 @@
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr"/>
+      <c r="I5" s="5" t="n"/>
+      <c r="J5" s="5" t="n"/>
+      <c r="K5" s="5" t="n"/>
+      <c r="L5" s="5" t="n"/>
+      <c r="M5" s="5" t="n"/>
     </row>
     <row r="6" ht="19.9" customHeight="1">
       <c r="A6" s="7">
@@ -1006,13 +1088,24 @@
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
-          <t>Dominio principal del proyecto</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Autoridad 51, spam bajo (18), 123 URLs indexadas</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr"/>
+      <c r="I6" s="27" t="n">
+        <v>51</v>
+      </c>
+      <c r="J6" s="25" t="n">
+        <v>123</v>
+      </c>
+      <c r="K6" s="25" t="n">
+        <v>9071</v>
+      </c>
+      <c r="L6" s="25" t="n">
+        <v>2802</v>
+      </c>
+      <c r="M6" s="25" t="n">
+        <v>18</v>
       </c>
     </row>
     <row r="7" ht="19.9" customHeight="1">
@@ -1046,10 +1139,15 @@
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>Subdominio ya marcado como Cancelar; no afecta renovación (depende de armoniapanama.com)</t>
+          <t>Subdominio ya marcado como Cancelar; no afecta la renovación (depende de armoniapanama.com)</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr"/>
+      <c r="I7" s="5" t="n"/>
+      <c r="J7" s="5" t="n"/>
+      <c r="K7" s="5" t="n"/>
+      <c r="L7" s="5" t="n"/>
+      <c r="M7" s="5" t="n"/>
     </row>
     <row r="8" ht="19.9" customHeight="1">
       <c r="A8" s="7">
@@ -1082,13 +1180,28 @@
       </c>
       <c r="G8" s="5" t="inlineStr">
         <is>
-          <t>Dominio principal del proyecto</t>
+          <t>Dominio principal activo, pero autoridad 0 y solo 2 URLs indexadas: problema de indexación a corregir</t>
         </is>
       </c>
       <c r="H8" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>spam alto: revisar/desautorizar enlaces</t>
+        </is>
+      </c>
+      <c r="I8" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="K8" s="25" t="n">
+        <v>2628</v>
+      </c>
+      <c r="L8" s="25" t="n">
+        <v>2498</v>
+      </c>
+      <c r="M8" s="26" t="n">
+        <v>54</v>
       </c>
     </row>
     <row r="9" ht="19.9" customHeight="1">
@@ -1122,13 +1235,24 @@
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>Dominio principal; sostiene 2 subdominios activos</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Autoridad 50, spam 26, sostiene subdominios activos</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="inlineStr"/>
+      <c r="I9" s="27" t="n">
+        <v>50</v>
+      </c>
+      <c r="J9" s="25" t="n">
+        <v>26</v>
+      </c>
+      <c r="K9" s="25" t="n">
+        <v>6236</v>
+      </c>
+      <c r="L9" s="25" t="n">
+        <v>2894</v>
+      </c>
+      <c r="M9" s="25" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="10" ht="19.9" customHeight="1">
@@ -1166,6 +1290,11 @@
         </is>
       </c>
       <c r="H10" s="5" t="inlineStr"/>
+      <c r="I10" s="5" t="n"/>
+      <c r="J10" s="5" t="n"/>
+      <c r="K10" s="5" t="n"/>
+      <c r="L10" s="5" t="n"/>
+      <c r="M10" s="5" t="n"/>
     </row>
     <row r="11" ht="19.9" customHeight="1">
       <c r="A11" s="7">
@@ -1202,6 +1331,11 @@
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr"/>
+      <c r="I11" s="5" t="n"/>
+      <c r="J11" s="5" t="n"/>
+      <c r="K11" s="5" t="n"/>
+      <c r="L11" s="5" t="n"/>
+      <c r="M11" s="5" t="n"/>
     </row>
     <row r="12" ht="19.9" customHeight="1">
       <c r="A12" s="7">
@@ -1234,13 +1368,28 @@
       </c>
       <c r="G12" s="5" t="inlineStr">
         <is>
-          <t>Dominio principal; sostiene 3 subdominios activos</t>
+          <t>Autoridad 42, 104 URLs indexadas, sostiene 3 subdominios activos</t>
         </is>
       </c>
       <c r="H12" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>spam alto: revisar/desautorizar enlaces</t>
+        </is>
+      </c>
+      <c r="I12" s="27" t="n">
+        <v>42</v>
+      </c>
+      <c r="J12" s="25" t="n">
+        <v>104</v>
+      </c>
+      <c r="K12" s="25" t="n">
+        <v>3240</v>
+      </c>
+      <c r="L12" s="25" t="n">
+        <v>2716</v>
+      </c>
+      <c r="M12" s="26" t="n">
+        <v>51</v>
       </c>
     </row>
     <row r="13" ht="19.9" customHeight="1">
@@ -1278,6 +1427,11 @@
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr"/>
+      <c r="I13" s="5" t="n"/>
+      <c r="J13" s="5" t="n"/>
+      <c r="K13" s="5" t="n"/>
+      <c r="L13" s="5" t="n"/>
+      <c r="M13" s="5" t="n"/>
     </row>
     <row r="14" ht="19.9" customHeight="1">
       <c r="A14" s="7">
@@ -1314,6 +1468,11 @@
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr"/>
+      <c r="I14" s="5" t="n"/>
+      <c r="J14" s="5" t="n"/>
+      <c r="K14" s="5" t="n"/>
+      <c r="L14" s="5" t="n"/>
+      <c r="M14" s="5" t="n"/>
     </row>
     <row r="15" ht="19.9" customHeight="1">
       <c r="A15" s="7">
@@ -1350,6 +1509,11 @@
         </is>
       </c>
       <c r="H15" s="5" t="inlineStr"/>
+      <c r="I15" s="5" t="n"/>
+      <c r="J15" s="5" t="n"/>
+      <c r="K15" s="5" t="n"/>
+      <c r="L15" s="5" t="n"/>
+      <c r="M15" s="5" t="n"/>
     </row>
     <row r="16" ht="19.9" customHeight="1">
       <c r="A16" s="7">
@@ -1382,13 +1546,24 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>Marca de centro comercial, .com.pa local</t>
-        </is>
-      </c>
-      <c r="H16" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Marca de centro comercial; perfil de enlaces pequeño pero propio (46 dominios ref.)</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="inlineStr"/>
+      <c r="I16" s="25" t="n">
+        <v>17</v>
+      </c>
+      <c r="J16" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="K16" s="25" t="n">
+        <v>59</v>
+      </c>
+      <c r="L16" s="25" t="n">
+        <v>46</v>
+      </c>
+      <c r="M16" s="25" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="17" ht="19.9" customHeight="1">
@@ -1422,13 +1597,30 @@
       </c>
       <c r="G17" s="5" t="inlineStr">
         <is>
-          <t>Dominio corporativo de la marca GLP</t>
+          <t>Dominio corporativo: autoridad 52, spam 5 (limpio). Sin resultado en site: de Google, verificar en Search Console</t>
         </is>
       </c>
       <c r="H17" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>site: sin resultados: confirmar en Search Console</t>
+        </is>
+      </c>
+      <c r="I17" s="27" t="n">
+        <v>52</v>
+      </c>
+      <c r="J17" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K17" s="25" t="n">
+        <v>12483</v>
+      </c>
+      <c r="L17" s="25" t="n">
+        <v>485</v>
+      </c>
+      <c r="M17" s="25" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="18" ht="19.9" customHeight="1">
@@ -1455,20 +1647,35 @@
           <t>Activo</t>
         </is>
       </c>
-      <c r="F18" s="23" t="inlineStr">
-        <is>
-          <t>Revisar</t>
+      <c r="F18" s="24" t="inlineStr">
+        <is>
+          <t>Dejar caducar</t>
         </is>
       </c>
       <c r="G18" s="5" t="inlineStr">
         <is>
-          <t>Secundario de GLP: dejar solo si tiene backlinks/tráfico; si no, 301 a glp.com.pa y caducar</t>
+          <t>Autoridad 8, spam 53, 10 URLs indexadas; sin valor propio. Redirigir 301 a glp.com.pa antes de soltar</t>
         </is>
       </c>
       <c r="H18" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>spam alto: revisar/desautorizar enlaces</t>
+        </is>
+      </c>
+      <c r="I18" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="J18" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="K18" s="25" t="n">
+        <v>2664</v>
+      </c>
+      <c r="L18" s="25" t="n">
+        <v>2513</v>
+      </c>
+      <c r="M18" s="26" t="n">
+        <v>53</v>
       </c>
     </row>
     <row r="19" ht="19.9" customHeight="1">
@@ -1502,13 +1709,28 @@
       </c>
       <c r="G19" s="5" t="inlineStr">
         <is>
-          <t>Secundario de GLP: dejar solo si tiene backlinks/tráfico; si no, 301 a glp.com.pa y caducar</t>
+          <t>Autoridad 43 pero casi todo el perfil es la red spam compartida (spam 51). Redirigir 301 a glp.com.pa y decidir</t>
         </is>
       </c>
       <c r="H19" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>spam alto: revisar/desautorizar enlaces</t>
+        </is>
+      </c>
+      <c r="I19" s="27" t="n">
+        <v>43</v>
+      </c>
+      <c r="J19" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="K19" s="25" t="n">
+        <v>3256</v>
+      </c>
+      <c r="L19" s="25" t="n">
+        <v>2850</v>
+      </c>
+      <c r="M19" s="26" t="n">
+        <v>51</v>
       </c>
     </row>
     <row r="20" ht="19.9" customHeight="1">
@@ -1542,13 +1764,30 @@
       </c>
       <c r="G20" s="5" t="inlineStr">
         <is>
-          <t>Dominio principal de Gran Terminal</t>
+          <t>Dominio principal, autoridad 19, spam 35. Sin resultado en site:, verificar indexación</t>
         </is>
       </c>
       <c r="H20" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>site: sin resultados: confirmar en Search Console</t>
+        </is>
+      </c>
+      <c r="I20" s="25" t="n">
+        <v>19</v>
+      </c>
+      <c r="J20" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K20" s="25" t="n">
+        <v>5161</v>
+      </c>
+      <c r="L20" s="25" t="n">
+        <v>2711</v>
+      </c>
+      <c r="M20" s="25" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="21" ht="19.9" customHeight="1">
@@ -1582,13 +1821,24 @@
       </c>
       <c r="G21" s="5" t="inlineStr">
         <is>
-          <t>Dominio principal del proyecto</t>
-        </is>
-      </c>
-      <c r="H21" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Autoridad 49, spam 19, 81 URLs indexadas</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr"/>
+      <c r="I21" s="27" t="n">
+        <v>49</v>
+      </c>
+      <c r="J21" s="25" t="n">
+        <v>81</v>
+      </c>
+      <c r="K21" s="25" t="n">
+        <v>7288</v>
+      </c>
+      <c r="L21" s="25" t="n">
+        <v>2832</v>
+      </c>
+      <c r="M21" s="25" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="22" ht="19.9" customHeight="1">
@@ -1622,13 +1872,24 @@
       </c>
       <c r="G22" s="5" t="inlineStr">
         <is>
-          <t>Dominio principal del proyecto</t>
-        </is>
-      </c>
-      <c r="H22" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Autoridad 46, spam 34, dominio principal</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="inlineStr"/>
+      <c r="I22" s="27" t="n">
+        <v>46</v>
+      </c>
+      <c r="J22" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="K22" s="25" t="n">
+        <v>5395</v>
+      </c>
+      <c r="L22" s="25" t="n">
+        <v>2718</v>
+      </c>
+      <c r="M22" s="25" t="n">
+        <v>34</v>
       </c>
     </row>
     <row r="23" ht="19.9" customHeight="1">
@@ -1662,13 +1923,30 @@
       </c>
       <c r="G23" s="5" t="inlineStr">
         <is>
-          <t>Marca de restaurante, dominio exacto</t>
+          <t>Marca de restaurante (dominio exacto). Autoridad 0 y sin indexar: revisar sitio</t>
         </is>
       </c>
       <c r="H23" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>site: sin resultados: confirmar en Search Console</t>
+        </is>
+      </c>
+      <c r="I23" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J23" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K23" s="25" t="n">
+        <v>2600</v>
+      </c>
+      <c r="L23" s="25" t="n">
+        <v>2470</v>
+      </c>
+      <c r="M23" s="25" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="24" ht="19.9" customHeight="1">
@@ -1702,13 +1980,24 @@
       </c>
       <c r="G24" s="5" t="inlineStr">
         <is>
-          <t>Dominio principal de la marca</t>
-        </is>
-      </c>
-      <c r="H24" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Mejor activo de la lista: autoridad 47, 6.6k dominios ref., ~300k URLs indexadas</t>
+        </is>
+      </c>
+      <c r="H24" s="5" t="inlineStr"/>
+      <c r="I24" s="27" t="n">
+        <v>47</v>
+      </c>
+      <c r="J24" s="25" t="n">
+        <v>307000</v>
+      </c>
+      <c r="K24" s="25" t="n">
+        <v>12310</v>
+      </c>
+      <c r="L24" s="25" t="n">
+        <v>6646</v>
+      </c>
+      <c r="M24" s="25" t="n">
+        <v>24</v>
       </c>
     </row>
     <row r="25" ht="19.9" customHeight="1">
@@ -1742,13 +2031,30 @@
       </c>
       <c r="G25" s="5" t="inlineStr">
         <is>
-          <t>Dominio principal del proyecto</t>
+          <t>Autoridad 43, dominio principal. Sin resultado en site:, verificar indexación</t>
         </is>
       </c>
       <c r="H25" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>site: sin resultados: confirmar en Search Console</t>
+        </is>
+      </c>
+      <c r="I25" s="27" t="n">
+        <v>43</v>
+      </c>
+      <c r="J25" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K25" s="25" t="n">
+        <v>3624</v>
+      </c>
+      <c r="L25" s="25" t="n">
+        <v>2555</v>
+      </c>
+      <c r="M25" s="25" t="n">
+        <v>41</v>
       </c>
     </row>
     <row r="26" ht="19.9" customHeight="1">
@@ -1786,6 +2092,11 @@
         </is>
       </c>
       <c r="H26" s="5" t="inlineStr"/>
+      <c r="I26" s="5" t="n"/>
+      <c r="J26" s="5" t="n"/>
+      <c r="K26" s="5" t="n"/>
+      <c r="L26" s="5" t="n"/>
+      <c r="M26" s="5" t="n"/>
     </row>
     <row r="27" ht="19.9" customHeight="1">
       <c r="A27" s="7">
@@ -1818,10 +2129,15 @@
       </c>
       <c r="G27" s="5" t="inlineStr">
         <is>
-          <t>Subdominio ya marcado como Cancelar; no afecta renovación (depende de oceanreefislands.com)</t>
+          <t>Subdominio ya marcado como Cancelar; no afecta la renovación (depende de oceanreefislands.com)</t>
         </is>
       </c>
       <c r="H27" s="5" t="inlineStr"/>
+      <c r="I27" s="5" t="n"/>
+      <c r="J27" s="5" t="n"/>
+      <c r="K27" s="5" t="n"/>
+      <c r="L27" s="5" t="n"/>
+      <c r="M27" s="5" t="n"/>
     </row>
     <row r="28" ht="19.9" customHeight="1">
       <c r="A28" s="7">
@@ -1854,10 +2170,15 @@
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Subdominio ya marcado como Cancelar; no afecta renovación (depende de oceanreefislands.com)</t>
+          <t>Subdominio ya marcado como Cancelar; no afecta la renovación (depende de oceanreefislands.com)</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr"/>
+      <c r="I28" s="5" t="n"/>
+      <c r="J28" s="5" t="n"/>
+      <c r="K28" s="5" t="n"/>
+      <c r="L28" s="5" t="n"/>
+      <c r="M28" s="5" t="n"/>
     </row>
     <row r="29" ht="19.9" customHeight="1">
       <c r="A29" s="7">
@@ -1890,10 +2211,15 @@
       </c>
       <c r="G29" s="5" t="inlineStr">
         <is>
-          <t>Subdominio ya marcado como Cancelar; no afecta renovación (depende de oceanreefislands.com)</t>
+          <t>Subdominio ya marcado como Cancelar; no afecta la renovación (depende de oceanreefislands.com)</t>
         </is>
       </c>
       <c r="H29" s="5" t="inlineStr"/>
+      <c r="I29" s="5" t="n"/>
+      <c r="J29" s="5" t="n"/>
+      <c r="K29" s="5" t="n"/>
+      <c r="L29" s="5" t="n"/>
+      <c r="M29" s="5" t="n"/>
     </row>
     <row r="30" ht="19.9" customHeight="1">
       <c r="A30" s="7">
@@ -1926,10 +2252,15 @@
       </c>
       <c r="G30" s="5" t="inlineStr">
         <is>
-          <t>Subdominio ya marcado como Cancelar; no afecta renovación (depende de oceanreefislands.com)</t>
+          <t>Subdominio ya marcado como Cancelar; no afecta la renovación (depende de oceanreefislands.com)</t>
         </is>
       </c>
       <c r="H30" s="5" t="inlineStr"/>
+      <c r="I30" s="5" t="n"/>
+      <c r="J30" s="5" t="n"/>
+      <c r="K30" s="5" t="n"/>
+      <c r="L30" s="5" t="n"/>
+      <c r="M30" s="5" t="n"/>
     </row>
     <row r="31" ht="19.9" customHeight="1">
       <c r="A31" s="7">
@@ -1962,13 +2293,24 @@
       </c>
       <c r="G31" s="5" t="inlineStr">
         <is>
-          <t>Dominio principal de Ocean Reef; sostiene subdominios activos</t>
-        </is>
-      </c>
-      <c r="H31" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Autoridad 51, spam 19, 153 URLs indexadas, sostiene subdominios activos</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr"/>
+      <c r="I31" s="27" t="n">
+        <v>51</v>
+      </c>
+      <c r="J31" s="25" t="n">
+        <v>153</v>
+      </c>
+      <c r="K31" s="25" t="n">
+        <v>8057</v>
+      </c>
+      <c r="L31" s="25" t="n">
+        <v>2800</v>
+      </c>
+      <c r="M31" s="25" t="n">
+        <v>19</v>
       </c>
     </row>
     <row r="32" ht="19.9" customHeight="1">
@@ -2002,13 +2344,24 @@
       </c>
       <c r="G32" s="5" t="inlineStr">
         <is>
-          <t>Marina: marca propia en .com.pa</t>
-        </is>
-      </c>
-      <c r="H32" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Spam bajo (14), 78 URLs indexadas, perfil de enlaces propio</t>
+        </is>
+      </c>
+      <c r="H32" s="5" t="inlineStr"/>
+      <c r="I32" s="25" t="n">
+        <v>37</v>
+      </c>
+      <c r="J32" s="25" t="n">
+        <v>78</v>
+      </c>
+      <c r="K32" s="25" t="n">
+        <v>220</v>
+      </c>
+      <c r="L32" s="25" t="n">
+        <v>52</v>
+      </c>
+      <c r="M32" s="25" t="n">
+        <v>14</v>
       </c>
     </row>
     <row r="33" ht="19.9" customHeight="1">
@@ -2042,13 +2395,28 @@
       </c>
       <c r="G33" s="5" t="inlineStr">
         <is>
-          <t>Dominio activo con marca propia</t>
+          <t>Dominio activo con marca propia, autoridad 0 y 4 URLs indexadas: reforzar contenido</t>
         </is>
       </c>
       <c r="H33" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>spam alto: revisar/desautorizar enlaces</t>
+        </is>
+      </c>
+      <c r="I33" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J33" s="25" t="n">
+        <v>4</v>
+      </c>
+      <c r="K33" s="25" t="n">
+        <v>2503</v>
+      </c>
+      <c r="L33" s="25" t="n">
+        <v>2375</v>
+      </c>
+      <c r="M33" s="26" t="n">
+        <v>54</v>
       </c>
     </row>
     <row r="34" ht="19.9" customHeight="1">
@@ -2086,6 +2454,11 @@
         </is>
       </c>
       <c r="H34" s="5" t="inlineStr"/>
+      <c r="I34" s="5" t="n"/>
+      <c r="J34" s="5" t="n"/>
+      <c r="K34" s="5" t="n"/>
+      <c r="L34" s="5" t="n"/>
+      <c r="M34" s="5" t="n"/>
     </row>
     <row r="35" ht="19.9" customHeight="1">
       <c r="A35" s="7">
@@ -2118,10 +2491,15 @@
       </c>
       <c r="G35" s="5" t="inlineStr">
         <is>
-          <t>Subdominio ya marcado como Cancelar; no afecta renovación (depende de oceanreefislands.com)</t>
+          <t>Subdominio ya marcado como Cancelar; no afecta la renovación (depende de oceanreefislands.com)</t>
         </is>
       </c>
       <c r="H35" s="5" t="inlineStr"/>
+      <c r="I35" s="5" t="n"/>
+      <c r="J35" s="5" t="n"/>
+      <c r="K35" s="5" t="n"/>
+      <c r="L35" s="5" t="n"/>
+      <c r="M35" s="5" t="n"/>
     </row>
     <row r="36" ht="19.9" customHeight="1">
       <c r="A36" s="7">
@@ -2154,10 +2532,15 @@
       </c>
       <c r="G36" s="5" t="inlineStr">
         <is>
-          <t>Subdominio ya marcado como Cancelar; no afecta renovación (depende de oceanreefislands.com)</t>
+          <t>Subdominio ya marcado como Cancelar; no afecta la renovación (depende de oceanreefislands.com)</t>
         </is>
       </c>
       <c r="H36" s="5" t="inlineStr"/>
+      <c r="I36" s="5" t="n"/>
+      <c r="J36" s="5" t="n"/>
+      <c r="K36" s="5" t="n"/>
+      <c r="L36" s="5" t="n"/>
+      <c r="M36" s="5" t="n"/>
     </row>
     <row r="37" ht="19.9" customHeight="1">
       <c r="A37" s="7">
@@ -2194,6 +2577,11 @@
         </is>
       </c>
       <c r="H37" s="5" t="inlineStr"/>
+      <c r="I37" s="5" t="n"/>
+      <c r="J37" s="5" t="n"/>
+      <c r="K37" s="5" t="n"/>
+      <c r="L37" s="5" t="n"/>
+      <c r="M37" s="5" t="n"/>
     </row>
     <row r="38" ht="19.9" customHeight="1">
       <c r="A38" s="7">
@@ -2226,13 +2614,28 @@
       </c>
       <c r="G38" s="5" t="inlineStr">
         <is>
-          <t>Estado Cancelar; microsite de campaña, redirigir si tuvo enlaces</t>
+          <t>En Cancelar; autoridad 0, 1 URL indexada, spam 54</t>
         </is>
       </c>
       <c r="H38" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>spam alto: revisar/desautorizar enlaces</t>
+        </is>
+      </c>
+      <c r="I38" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J38" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="K38" s="25" t="n">
+        <v>2506</v>
+      </c>
+      <c r="L38" s="25" t="n">
+        <v>2377</v>
+      </c>
+      <c r="M38" s="26" t="n">
+        <v>54</v>
       </c>
     </row>
     <row r="39" ht="19.9" customHeight="1">
@@ -2266,13 +2669,24 @@
       </c>
       <c r="G39" s="5" t="inlineStr">
         <is>
-          <t>Dominio principal de Oceana</t>
-        </is>
-      </c>
-      <c r="H39" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Autoridad 51, spam 20, 60 URLs indexadas</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr"/>
+      <c r="I39" s="27" t="n">
+        <v>51</v>
+      </c>
+      <c r="J39" s="25" t="n">
+        <v>60</v>
+      </c>
+      <c r="K39" s="25" t="n">
+        <v>8589</v>
+      </c>
+      <c r="L39" s="25" t="n">
+        <v>2752</v>
+      </c>
+      <c r="M39" s="25" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="40" ht="19.9" customHeight="1">
@@ -2306,10 +2720,15 @@
       </c>
       <c r="G40" s="5" t="inlineStr">
         <is>
-          <t>Subdominio ya marcado como Cancelar; no afecta renovación (depende de oceanasantamaria.com)</t>
+          <t>Subdominio ya marcado como Cancelar; no afecta la renovación (depende de oceanasantamaria.com)</t>
         </is>
       </c>
       <c r="H40" s="5" t="inlineStr"/>
+      <c r="I40" s="5" t="n"/>
+      <c r="J40" s="5" t="n"/>
+      <c r="K40" s="5" t="n"/>
+      <c r="L40" s="5" t="n"/>
+      <c r="M40" s="5" t="n"/>
     </row>
     <row r="41" ht="19.9" customHeight="1">
       <c r="A41" s="7">
@@ -2342,10 +2761,15 @@
       </c>
       <c r="G41" s="5" t="inlineStr">
         <is>
-          <t>Subdominio ya marcado como Cancelar; no afecta renovación (depende de oceanasantamaria.com)</t>
+          <t>Subdominio ya marcado como Cancelar; no afecta la renovación (depende de oceanasantamaria.com)</t>
         </is>
       </c>
       <c r="H41" s="5" t="inlineStr"/>
+      <c r="I41" s="5" t="n"/>
+      <c r="J41" s="5" t="n"/>
+      <c r="K41" s="5" t="n"/>
+      <c r="L41" s="5" t="n"/>
+      <c r="M41" s="5" t="n"/>
     </row>
     <row r="42" ht="19.9" customHeight="1">
       <c r="A42" s="7">
@@ -2378,13 +2802,28 @@
       </c>
       <c r="G42" s="5" t="inlineStr">
         <is>
-          <t>Estado Cancelar; solapa con panamaviejoresidences.com</t>
+          <t>En Cancelar; autoridad 3, spam 53, solapa con panamaviejoresidences.com</t>
         </is>
       </c>
       <c r="H42" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>spam alto: revisar/desautorizar enlaces</t>
+        </is>
+      </c>
+      <c r="I42" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="J42" s="25" t="n">
+        <v>24</v>
+      </c>
+      <c r="K42" s="25" t="n">
+        <v>2533</v>
+      </c>
+      <c r="L42" s="25" t="n">
+        <v>2397</v>
+      </c>
+      <c r="M42" s="26" t="n">
+        <v>53</v>
       </c>
     </row>
     <row r="43" ht="19.9" customHeight="1">
@@ -2418,13 +2857,24 @@
       </c>
       <c r="G43" s="5" t="inlineStr">
         <is>
-          <t>Dominio principal activo del proyecto</t>
-        </is>
-      </c>
-      <c r="H43" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Autoridad 50, spam 23, 150 URLs indexadas</t>
+        </is>
+      </c>
+      <c r="H43" s="5" t="inlineStr"/>
+      <c r="I43" s="27" t="n">
+        <v>50</v>
+      </c>
+      <c r="J43" s="25" t="n">
+        <v>150</v>
+      </c>
+      <c r="K43" s="25" t="n">
+        <v>6605</v>
+      </c>
+      <c r="L43" s="25" t="n">
+        <v>2743</v>
+      </c>
+      <c r="M43" s="25" t="n">
+        <v>23</v>
       </c>
     </row>
     <row r="44" ht="19.9" customHeight="1">
@@ -2458,13 +2908,24 @@
       </c>
       <c r="G44" s="5" t="inlineStr">
         <is>
-          <t>Estado Cancelar; microsite de fase, canibaliza el principal</t>
-        </is>
-      </c>
-      <c r="H44" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>En Cancelar; autoridad 5, 2 URLs indexadas, spam 44</t>
+        </is>
+      </c>
+      <c r="H44" s="5" t="inlineStr"/>
+      <c r="I44" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="J44" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="K44" s="25" t="n">
+        <v>2647</v>
+      </c>
+      <c r="L44" s="25" t="n">
+        <v>2512</v>
+      </c>
+      <c r="M44" s="25" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="45" ht="19.9" customHeight="1">
@@ -2491,20 +2952,31 @@
           <t>Cancelar</t>
         </is>
       </c>
-      <c r="F45" s="24" t="inlineStr">
-        <is>
-          <t>Dejar caducar</t>
+      <c r="F45" s="23" t="inlineStr">
+        <is>
+          <t>Revisar</t>
         </is>
       </c>
       <c r="G45" s="5" t="inlineStr">
         <is>
-          <t>Estado Cancelar; microsite de campaña</t>
-        </is>
-      </c>
-      <c r="H45" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>En Cancelar pero tiene autoridad 39 y 427 URLs indexadas: redirigir 301 a playacaracolresidences.com antes de soltar</t>
+        </is>
+      </c>
+      <c r="H45" s="5" t="inlineStr"/>
+      <c r="I45" s="25" t="n">
+        <v>39</v>
+      </c>
+      <c r="J45" s="25" t="n">
+        <v>427</v>
+      </c>
+      <c r="K45" s="25" t="n">
+        <v>3879</v>
+      </c>
+      <c r="L45" s="25" t="n">
+        <v>2599</v>
+      </c>
+      <c r="M45" s="25" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="46" ht="19.9" customHeight="1">
@@ -2538,13 +3010,24 @@
       </c>
       <c r="G46" s="5" t="inlineStr">
         <is>
-          <t>Estado Cancelar; microsite de campaña</t>
-        </is>
-      </c>
-      <c r="H46" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>En Cancelar; autoridad 0, 3 URLs indexadas, spam 44</t>
+        </is>
+      </c>
+      <c r="H46" s="5" t="inlineStr"/>
+      <c r="I46" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J46" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="K46" s="25" t="n">
+        <v>2601</v>
+      </c>
+      <c r="L46" s="25" t="n">
+        <v>2477</v>
+      </c>
+      <c r="M46" s="25" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="47" ht="19.9" customHeight="1">
@@ -2582,6 +3065,11 @@
         </is>
       </c>
       <c r="H47" s="5" t="inlineStr"/>
+      <c r="I47" s="5" t="n"/>
+      <c r="J47" s="5" t="n"/>
+      <c r="K47" s="5" t="n"/>
+      <c r="L47" s="5" t="n"/>
+      <c r="M47" s="5" t="n"/>
     </row>
     <row r="48" ht="19.9" customHeight="1">
       <c r="A48" s="7">
@@ -2614,13 +3102,28 @@
       </c>
       <c r="G48" s="5" t="inlineStr">
         <is>
-          <t>Activo; marca + intención de descubrimiento</t>
+          <t>Activo, pero autoridad 0 y 1 URL indexada: confirmar que realmente se usa</t>
         </is>
       </c>
       <c r="H48" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>spam alto: revisar/desautorizar enlaces</t>
+        </is>
+      </c>
+      <c r="I48" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J48" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="K48" s="25" t="n">
+        <v>2624</v>
+      </c>
+      <c r="L48" s="25" t="n">
+        <v>2497</v>
+      </c>
+      <c r="M48" s="26" t="n">
+        <v>54</v>
       </c>
     </row>
     <row r="49" ht="19.9" customHeight="1">
@@ -2654,10 +3157,15 @@
       </c>
       <c r="G49" s="5" t="inlineStr">
         <is>
-          <t>Subdominio ya marcado como Cancelar; no afecta renovación (depende de playacaracolresidences.com)</t>
+          <t>Subdominio ya marcado como Cancelar; no afecta la renovación (depende de playacaracolresidences.com)</t>
         </is>
       </c>
       <c r="H49" s="5" t="inlineStr"/>
+      <c r="I49" s="5" t="n"/>
+      <c r="J49" s="5" t="n"/>
+      <c r="K49" s="5" t="n"/>
+      <c r="L49" s="5" t="n"/>
+      <c r="M49" s="5" t="n"/>
     </row>
     <row r="50" ht="19.9" customHeight="1">
       <c r="A50" s="7">
@@ -2683,20 +3191,37 @@
           <t>Activo</t>
         </is>
       </c>
-      <c r="F50" s="23" t="inlineStr">
-        <is>
-          <t>Revisar</t>
+      <c r="F50" s="24" t="inlineStr">
+        <is>
+          <t>Dejar caducar</t>
         </is>
       </c>
       <c r="G50" s="5" t="inlineStr">
         <is>
-          <t>Activo pero sin marca Playa Caracol en el dominio: validar tráfico propio</t>
+          <t>Autoridad 0, 28 backlinks, spam 62 (el más alto), sin indexar y sin marca en el dominio</t>
         </is>
       </c>
       <c r="H50" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>site: sin resultados: confirmar en Search Console; spam alto: revisar/desautorizar enlaces</t>
+        </is>
+      </c>
+      <c r="I50" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J50" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K50" s="25" t="n">
+        <v>28</v>
+      </c>
+      <c r="L50" s="25" t="n">
+        <v>25</v>
+      </c>
+      <c r="M50" s="26" t="n">
+        <v>62</v>
       </c>
     </row>
     <row r="51" ht="19.9" customHeight="1">
@@ -2730,13 +3255,28 @@
       </c>
       <c r="G51" s="5" t="inlineStr">
         <is>
-          <t>Estado Cancelar; dominio de captación genérico</t>
+          <t>En Cancelar; autoridad 0, 2 URLs indexadas, spam 54</t>
         </is>
       </c>
       <c r="H51" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>spam alto: revisar/desautorizar enlaces</t>
+        </is>
+      </c>
+      <c r="I51" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J51" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="K51" s="25" t="n">
+        <v>2631</v>
+      </c>
+      <c r="L51" s="25" t="n">
+        <v>2495</v>
+      </c>
+      <c r="M51" s="26" t="n">
+        <v>54</v>
       </c>
     </row>
     <row r="52" ht="19.9" customHeight="1">
@@ -2774,6 +3314,11 @@
         </is>
       </c>
       <c r="H52" s="5" t="inlineStr"/>
+      <c r="I52" s="5" t="n"/>
+      <c r="J52" s="5" t="n"/>
+      <c r="K52" s="5" t="n"/>
+      <c r="L52" s="5" t="n"/>
+      <c r="M52" s="5" t="n"/>
     </row>
     <row r="53" ht="19.9" customHeight="1">
       <c r="A53" s="7">
@@ -2806,13 +3351,24 @@
       </c>
       <c r="G53" s="5" t="inlineStr">
         <is>
-          <t>Activo; sostiene subdominio international</t>
-        </is>
-      </c>
-      <c r="H53" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Autoridad 43, 220 URLs indexadas, sostiene subdominio activo</t>
+        </is>
+      </c>
+      <c r="H53" s="5" t="inlineStr"/>
+      <c r="I53" s="27" t="n">
+        <v>43</v>
+      </c>
+      <c r="J53" s="25" t="n">
+        <v>220</v>
+      </c>
+      <c r="K53" s="25" t="n">
+        <v>4405</v>
+      </c>
+      <c r="L53" s="25" t="n">
+        <v>2564</v>
+      </c>
+      <c r="M53" s="25" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="54" ht="19.9" customHeight="1">
@@ -2846,13 +3402,24 @@
       </c>
       <c r="G54" s="5" t="inlineStr">
         <is>
-          <t>Dominio principal con marca; presente en listados de terceros</t>
-        </is>
-      </c>
-      <c r="H54" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Autoridad 48, spam 26, 112 URLs indexadas</t>
+        </is>
+      </c>
+      <c r="H54" s="5" t="inlineStr"/>
+      <c r="I54" s="27" t="n">
+        <v>48</v>
+      </c>
+      <c r="J54" s="25" t="n">
+        <v>112</v>
+      </c>
+      <c r="K54" s="25" t="n">
+        <v>5733</v>
+      </c>
+      <c r="L54" s="25" t="n">
+        <v>2847</v>
+      </c>
+      <c r="M54" s="25" t="n">
+        <v>26</v>
       </c>
     </row>
     <row r="55" ht="19.9" customHeight="1">
@@ -2886,13 +3453,24 @@
       </c>
       <c r="G55" s="5" t="inlineStr">
         <is>
-          <t>Dominio principal activo; sostiene subdominio</t>
-        </is>
-      </c>
-      <c r="H55" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Dominio principal activo, autoridad 12, sostiene subdominio</t>
+        </is>
+      </c>
+      <c r="H55" s="5" t="inlineStr"/>
+      <c r="I55" s="25" t="n">
+        <v>12</v>
+      </c>
+      <c r="J55" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="K55" s="25" t="n">
+        <v>2552</v>
+      </c>
+      <c r="L55" s="25" t="n">
+        <v>2415</v>
+      </c>
+      <c r="M55" s="25" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="56" ht="19.9" customHeight="1">
@@ -2926,13 +3504,28 @@
       </c>
       <c r="G56" s="5" t="inlineStr">
         <is>
-          <t>Estado Cancelar; microsite de torre</t>
+          <t>En Cancelar; autoridad 0, 2 URLs indexadas, spam 54</t>
         </is>
       </c>
       <c r="H56" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>spam alto: revisar/desautorizar enlaces</t>
+        </is>
+      </c>
+      <c r="I56" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J56" s="25" t="n">
+        <v>2</v>
+      </c>
+      <c r="K56" s="25" t="n">
+        <v>2570</v>
+      </c>
+      <c r="L56" s="25" t="n">
+        <v>2446</v>
+      </c>
+      <c r="M56" s="26" t="n">
+        <v>54</v>
       </c>
     </row>
     <row r="57" ht="19.9" customHeight="1">
@@ -2966,13 +3559,24 @@
       </c>
       <c r="G57" s="5" t="inlineStr">
         <is>
-          <t>Activo; microsite de torre vigente</t>
-        </is>
-      </c>
-      <c r="H57" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Activo (microsite de torre vigente), aunque con autoridad 0 y 1 URL indexada</t>
+        </is>
+      </c>
+      <c r="H57" s="5" t="inlineStr"/>
+      <c r="I57" s="25" t="n">
+        <v>0</v>
+      </c>
+      <c r="J57" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="K57" s="25" t="n">
+        <v>2522</v>
+      </c>
+      <c r="L57" s="25" t="n">
+        <v>2399</v>
+      </c>
+      <c r="M57" s="25" t="n">
+        <v>44</v>
       </c>
     </row>
     <row r="58" ht="19.9" customHeight="1">
@@ -3006,13 +3610,28 @@
       </c>
       <c r="G58" s="5" t="inlineStr">
         <is>
-          <t>Estado Cancelar; microsite de torre</t>
+          <t>En Cancelar; autoridad 12, 5 URLs indexadas, spam 54</t>
         </is>
       </c>
       <c r="H58" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>spam alto: revisar/desautorizar enlaces</t>
+        </is>
+      </c>
+      <c r="I58" s="25" t="n">
+        <v>12</v>
+      </c>
+      <c r="J58" s="25" t="n">
+        <v>5</v>
+      </c>
+      <c r="K58" s="25" t="n">
+        <v>2585</v>
+      </c>
+      <c r="L58" s="25" t="n">
+        <v>2451</v>
+      </c>
+      <c r="M58" s="26" t="n">
+        <v>54</v>
       </c>
     </row>
     <row r="59" ht="19.9" customHeight="1">
@@ -3039,20 +3658,31 @@
           <t>Cancelar</t>
         </is>
       </c>
-      <c r="F59" s="23" t="inlineStr">
-        <is>
-          <t>Revisar</t>
+      <c r="F59" s="22" t="inlineStr">
+        <is>
+          <t>Dejar</t>
         </is>
       </c>
       <c r="G59" s="5" t="inlineStr">
         <is>
-          <t>Estado Cancelar pero es el dominio exacto de marca (.com.pa): revisar backlinks antes de soltar; lo normal es 301 a playadoradaresidences.com</t>
-        </is>
-      </c>
-      <c r="H59" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>En Cancelar pero es el mejor activo del proyecto: autoridad 49, spam 5, 521 dominios ref. propios, 256 URLs indexadas. Mantener o 301 a playadoradaresidences.com</t>
+        </is>
+      </c>
+      <c r="H59" s="5" t="inlineStr"/>
+      <c r="I59" s="27" t="n">
+        <v>49</v>
+      </c>
+      <c r="J59" s="25" t="n">
+        <v>256</v>
+      </c>
+      <c r="K59" s="25" t="n">
+        <v>4787</v>
+      </c>
+      <c r="L59" s="25" t="n">
+        <v>521</v>
+      </c>
+      <c r="M59" s="25" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="60" ht="19.9" customHeight="1">
@@ -3086,13 +3716,28 @@
       </c>
       <c r="G60" s="5" t="inlineStr">
         <is>
-          <t>Dominio principal activo</t>
+          <t>Dominio activo del proyecto; autoridad 3 y 6 URLs indexadas, depende de redirigir/enlazar desde playadorada.com.pa</t>
         </is>
       </c>
       <c r="H60" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>spam alto: revisar/desautorizar enlaces</t>
+        </is>
+      </c>
+      <c r="I60" s="25" t="n">
+        <v>3</v>
+      </c>
+      <c r="J60" s="25" t="n">
+        <v>6</v>
+      </c>
+      <c r="K60" s="25" t="n">
+        <v>2567</v>
+      </c>
+      <c r="L60" s="25" t="n">
+        <v>2428</v>
+      </c>
+      <c r="M60" s="26" t="n">
+        <v>53</v>
       </c>
     </row>
     <row r="61" ht="19.9" customHeight="1">
@@ -3126,10 +3771,15 @@
       </c>
       <c r="G61" s="5" t="inlineStr">
         <is>
-          <t>Subdominio ya marcado como Cancelar; no afecta renovación (depende de playadoradaresidences.com)</t>
+          <t>Subdominio ya marcado como Cancelar; no afecta la renovación (depende de playadoradaresidences.com)</t>
         </is>
       </c>
       <c r="H61" s="5" t="inlineStr"/>
+      <c r="I61" s="5" t="n"/>
+      <c r="J61" s="5" t="n"/>
+      <c r="K61" s="5" t="n"/>
+      <c r="L61" s="5" t="n"/>
+      <c r="M61" s="5" t="n"/>
     </row>
     <row r="62" ht="19.9" customHeight="1">
       <c r="A62" s="7">
@@ -3166,6 +3816,11 @@
         </is>
       </c>
       <c r="H62" s="5" t="inlineStr"/>
+      <c r="I62" s="5" t="n"/>
+      <c r="J62" s="5" t="n"/>
+      <c r="K62" s="5" t="n"/>
+      <c r="L62" s="5" t="n"/>
+      <c r="M62" s="5" t="n"/>
     </row>
     <row r="63" ht="19.9" customHeight="1">
       <c r="A63" s="7">
@@ -3198,13 +3853,24 @@
       </c>
       <c r="G63" s="5" t="inlineStr">
         <is>
-          <t>Dominio principal; sostiene subdominio</t>
-        </is>
-      </c>
-      <c r="H63" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Autoridad 44, spam 35, sostiene subdominio</t>
+        </is>
+      </c>
+      <c r="H63" s="5" t="inlineStr"/>
+      <c r="I63" s="27" t="n">
+        <v>44</v>
+      </c>
+      <c r="J63" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="K63" s="25" t="n">
+        <v>4487</v>
+      </c>
+      <c r="L63" s="25" t="n">
+        <v>2516</v>
+      </c>
+      <c r="M63" s="25" t="n">
+        <v>35</v>
       </c>
     </row>
     <row r="64" ht="19.9" customHeight="1">
@@ -3238,12 +3904,31 @@
       </c>
       <c r="G64" s="5" t="inlineStr">
         <is>
-          <t>Dominio activo, .com.pa local</t>
-        </is>
-      </c>
-      <c r="H64" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
+          <t>Dominio activo; DataForSEO no tiene datos de backlinks (perfil prácticamente vacío), 1 URL indexada</t>
+        </is>
+      </c>
+      <c r="H64" s="5" t="inlineStr"/>
+      <c r="I64" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="J64" s="25" t="n">
+        <v>1</v>
+      </c>
+      <c r="K64" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="L64" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="M64" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
     </row>
@@ -3278,13 +3963,24 @@
       </c>
       <c r="G65" s="5" t="inlineStr">
         <is>
-          <t>Dominio activo, nombre corto de marca (.com.pa)</t>
-        </is>
-      </c>
-      <c r="H65" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Nombre corto de marca; autoridad 14, 81 dominios ref. propios</t>
+        </is>
+      </c>
+      <c r="H65" s="5" t="inlineStr"/>
+      <c r="I65" s="25" t="n">
+        <v>14</v>
+      </c>
+      <c r="J65" s="25" t="n">
+        <v>10</v>
+      </c>
+      <c r="K65" s="25" t="n">
+        <v>153</v>
+      </c>
+      <c r="L65" s="25" t="n">
+        <v>81</v>
+      </c>
+      <c r="M65" s="25" t="n">
+        <v>46</v>
       </c>
     </row>
     <row r="66" ht="19.9" customHeight="1">
@@ -3318,13 +4014,24 @@
       </c>
       <c r="G66" s="5" t="inlineStr">
         <is>
-          <t>Dominio activo con marca</t>
-        </is>
-      </c>
-      <c r="H66" s="5" t="inlineStr">
-        <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>Autoridad 53, spam 3 (el más limpio), 408 dominios ref. propios</t>
+        </is>
+      </c>
+      <c r="H66" s="5" t="inlineStr"/>
+      <c r="I66" s="27" t="n">
+        <v>53</v>
+      </c>
+      <c r="J66" s="25" t="n">
+        <v>51</v>
+      </c>
+      <c r="K66" s="25" t="n">
+        <v>10047</v>
+      </c>
+      <c r="L66" s="25" t="n">
+        <v>408</v>
+      </c>
+      <c r="M66" s="25" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="67" ht="19.9" customHeight="1">
@@ -3358,10 +4065,15 @@
       </c>
       <c r="G67" s="5" t="inlineStr">
         <is>
-          <t>Subdominio ya marcado como Cancelar; no afecta renovación (depende de ventuhomtel.com)</t>
+          <t>Subdominio ya marcado como Cancelar; no afecta la renovación (depende de ventuhomtel.com)</t>
         </is>
       </c>
       <c r="H67" s="5" t="inlineStr"/>
+      <c r="I67" s="5" t="n"/>
+      <c r="J67" s="5" t="n"/>
+      <c r="K67" s="5" t="n"/>
+      <c r="L67" s="5" t="n"/>
+      <c r="M67" s="5" t="n"/>
     </row>
     <row r="68" ht="19.9" customHeight="1">
       <c r="A68" s="7">
@@ -3394,10 +4106,15 @@
       </c>
       <c r="G68" s="5" t="inlineStr">
         <is>
-          <t>Subdominio ya marcado como Cancelar; no afecta renovación (depende de ventuhomtel.com)</t>
+          <t>Subdominio ya marcado como Cancelar; no afecta la renovación (depende de ventuhomtel.com)</t>
         </is>
       </c>
       <c r="H68" s="5" t="inlineStr"/>
+      <c r="I68" s="5" t="n"/>
+      <c r="J68" s="5" t="n"/>
+      <c r="K68" s="5" t="n"/>
+      <c r="L68" s="5" t="n"/>
+      <c r="M68" s="5" t="n"/>
     </row>
     <row r="69" ht="19.9" customHeight="1">
       <c r="A69" s="7">
@@ -3430,10 +4147,15 @@
       </c>
       <c r="G69" s="5" t="inlineStr">
         <is>
-          <t>Subdominio ya marcado como Cancelar; no afecta renovación (depende de ventuhomtel.com)</t>
+          <t>Subdominio ya marcado como Cancelar; no afecta la renovación (depende de ventuhomtel.com)</t>
         </is>
       </c>
       <c r="H69" s="5" t="inlineStr"/>
+      <c r="I69" s="5" t="n"/>
+      <c r="J69" s="5" t="n"/>
+      <c r="K69" s="5" t="n"/>
+      <c r="L69" s="5" t="n"/>
+      <c r="M69" s="5" t="n"/>
     </row>
     <row r="70" ht="19.9" customHeight="1">
       <c r="A70" s="7">
@@ -3466,13 +4188,28 @@
       </c>
       <c r="G70" s="5" t="inlineStr">
         <is>
-          <t>Dominio principal; sostiene subdominios</t>
+          <t>Dominio principal activo, autoridad 17, 70 URLs indexadas, sostiene subdominios</t>
         </is>
       </c>
       <c r="H70" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>spam alto: revisar/desautorizar enlaces</t>
+        </is>
+      </c>
+      <c r="I70" s="25" t="n">
+        <v>17</v>
+      </c>
+      <c r="J70" s="25" t="n">
+        <v>70</v>
+      </c>
+      <c r="K70" s="25" t="n">
+        <v>2548</v>
+      </c>
+      <c r="L70" s="25" t="n">
+        <v>2412</v>
+      </c>
+      <c r="M70" s="26" t="n">
+        <v>53</v>
       </c>
     </row>
     <row r="71" ht="19.9" customHeight="1">
@@ -3506,13 +4243,30 @@
       </c>
       <c r="G71" s="5" t="inlineStr">
         <is>
-          <t>Marca de centro comercial, .com.pa local</t>
+          <t>Marca de centro comercial; 262 dominios ref. propios, autoridad 19. Sin resultado en site:, verificar</t>
         </is>
       </c>
       <c r="H71" s="5" t="inlineStr">
         <is>
-          <t>Indexación (GSC/site:), backlinks y dominios de referencia (Ahrefs/Semrush)</t>
-        </is>
+          <t>site: sin resultados: confirmar en Search Console</t>
+        </is>
+      </c>
+      <c r="I71" s="25" t="n">
+        <v>19</v>
+      </c>
+      <c r="J71" s="25" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="K71" s="25" t="n">
+        <v>422</v>
+      </c>
+      <c r="L71" s="25" t="n">
+        <v>262</v>
+      </c>
+      <c r="M71" s="25" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="74" ht="18.75" customHeight="1">
@@ -4286,4 +5040,106 @@
     <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="28" t="inlineStr">
+        <is>
+          <t>Fuente</t>
+        </is>
+      </c>
+      <c r="B1" s="29" t="inlineStr">
+        <is>
+          <t>DataForSEO (Backlinks API + SERP API), consultado 2026-10-24. Solo dominios raíz; los subdominios heredan la decisión de su raíz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="28" t="inlineStr">
+        <is>
+          <t>Autoridad (0-100)</t>
+        </is>
+      </c>
+      <c r="B2" s="29" t="inlineStr">
+        <is>
+          <t>Domain rank de DataForSEO, calculado a partir de backlinks (escala 0-100). No es el DA de Moz ni el DR de Ahrefs, pero es comparable entre estos dominios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="28" t="inlineStr">
+        <is>
+          <t>URLs indexadas</t>
+        </is>
+      </c>
+      <c r="B3" s="29" t="inlineStr">
+        <is>
+          <t>Resultados estimados de Google para site:dominio (Panamá, español). Es una estimación aproximada; "—" = Google no devolvió resultados, confirmar en Search Console.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="28" t="inlineStr">
+        <is>
+          <t>Backlinks / Dominios de referencia</t>
+        </is>
+      </c>
+      <c r="B4" s="29" t="inlineStr">
+        <is>
+          <t>Totales de DataForSEO (dominios de referencia = dominios principales únicos).</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="28" t="inlineStr">
+        <is>
+          <t>Spam score</t>
+        </is>
+      </c>
+      <c r="B5" s="29" t="inlineStr">
+        <is>
+          <t>0-100 de DataForSEO. 50 o más = alto.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="28" t="inlineStr">
+        <is>
+          <t>Hallazgo importante</t>
+        </is>
+      </c>
+      <c r="B6" s="29" t="inlineStr">
+        <is>
+          <t>Unos 35 dominios del inventario comparten entre 2.400 y 2.900 dominios de referencia con spam score 44-54. Es el mismo bloque de enlaces basura apuntando a casi todo el hosting. Inflan "Backlinks" y "Dominios de referencia" pero no aportan autoridad: el valor real está en los dominios con autoridad alta y spam bajo (metrolibre.com, glp.com.pa, playadorada.com.pa, supremestorage.net, oceanreefislands.com, armoniapanama.com).</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="28" t="inlineStr">
+        <is>
+          <t>Criterio de decisión</t>
+        </is>
+      </c>
+      <c r="B7" s="29" t="inlineStr">
+        <is>
+          <t>Dejar = marca/dominio principal o con autoridad y spam razonable. Dejar caducar = Cancelar o sin marca, con autoridad cercana a 0, casi sin indexar. Revisar = tiene autoridad o indexación: redirigir 301 al dominio principal antes de soltar.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>